<commit_message>
feat(tms): implement vehicle template export functionality and update repositories
</commit_message>
<xml_diff>
--- a/first-mile/src/main/resources/excel/vehicle_template.xlsx
+++ b/first-mile/src/main/resources/excel/vehicle_template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Desktop\hanh chinh vn\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Desktop\DATN\Serp\first-mile\src\main\resources\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EA77162-C5A5-4AC6-881D-66071764A9F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19CE624A-ABE2-455C-8573-55293009A50A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="VEHICLE" sheetId="1" r:id="rId1"/>
@@ -476,7 +476,7 @@
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="4">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{F893D5E3-AFB9-4F2A-808F-A47560C6602F}">
           <x14:formula1>
             <xm:f>Unit!$B$2:$B$3</xm:f>
@@ -488,6 +488,18 @@
             <xm:f>Unit!$A$2:$A$6</xm:f>
           </x14:formula1>
           <xm:sqref>H2:H1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{A5818E3A-48D5-4FEF-95D1-C1718E835248}">
+          <x14:formula1>
+            <xm:f>Unit!$C$2:$C$40068</xm:f>
+          </x14:formula1>
+          <xm:sqref>E2:E1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{3BFF862F-9841-4542-9621-B0E6D59B3320}">
+          <x14:formula1>
+            <xm:f>Unit!$D$2:$D$43169</xm:f>
+          </x14:formula1>
+          <xm:sqref>F2:F1048576</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>